<commit_message>
Update PSX indices data
</commit_message>
<xml_diff>
--- a/data/psx_indices_history.xlsx
+++ b/data/psx_indices_history.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,7 +491,7 @@
         </is>
       </c>
       <c r="H2" s="1" t="n">
-        <v>46196.72965276291</v>
+        <v>46196.7296527662</v>
       </c>
     </row>
     <row r="3">
@@ -523,7 +523,7 @@
         </is>
       </c>
       <c r="H3" s="1" t="n">
-        <v>46196.72965276291</v>
+        <v>46196.7296527662</v>
       </c>
     </row>
     <row r="4">
@@ -555,7 +555,7 @@
         </is>
       </c>
       <c r="H4" s="1" t="n">
-        <v>46196.72965276291</v>
+        <v>46196.7296527662</v>
       </c>
     </row>
     <row r="5">
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="H5" s="1" t="n">
-        <v>46196.72965276291</v>
+        <v>46196.7296527662</v>
       </c>
     </row>
     <row r="6">
@@ -619,7 +619,7 @@
         </is>
       </c>
       <c r="H6" s="1" t="n">
-        <v>46196.72965276291</v>
+        <v>46196.7296527662</v>
       </c>
     </row>
     <row r="7">
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="H7" s="1" t="n">
-        <v>46196.72965276291</v>
+        <v>46196.7296527662</v>
       </c>
     </row>
     <row r="8">
@@ -683,7 +683,7 @@
         </is>
       </c>
       <c r="H8" s="1" t="n">
-        <v>46196.72965276291</v>
+        <v>46196.7296527662</v>
       </c>
     </row>
     <row r="9">
@@ -715,7 +715,7 @@
         </is>
       </c>
       <c r="H9" s="1" t="n">
-        <v>46196.72965276291</v>
+        <v>46196.7296527662</v>
       </c>
     </row>
     <row r="10">
@@ -747,7 +747,7 @@
         </is>
       </c>
       <c r="H10" s="1" t="n">
-        <v>46196.72965276291</v>
+        <v>46196.7296527662</v>
       </c>
     </row>
     <row r="11">
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="H11" s="1" t="n">
-        <v>46196.72965276291</v>
+        <v>46196.7296527662</v>
       </c>
     </row>
     <row r="12">
@@ -811,7 +811,7 @@
         </is>
       </c>
       <c r="H12" s="1" t="n">
-        <v>46196.72965276291</v>
+        <v>46196.7296527662</v>
       </c>
     </row>
     <row r="13">
@@ -843,7 +843,7 @@
         </is>
       </c>
       <c r="H13" s="1" t="n">
-        <v>46196.72965276291</v>
+        <v>46196.7296527662</v>
       </c>
     </row>
     <row r="14">
@@ -875,7 +875,7 @@
         </is>
       </c>
       <c r="H14" s="1" t="n">
-        <v>46196.72965276291</v>
+        <v>46196.7296527662</v>
       </c>
     </row>
     <row r="15">
@@ -907,7 +907,7 @@
         </is>
       </c>
       <c r="H15" s="1" t="n">
-        <v>46196.72965276291</v>
+        <v>46196.7296527662</v>
       </c>
     </row>
     <row r="16">
@@ -939,7 +939,7 @@
         </is>
       </c>
       <c r="H16" s="1" t="n">
-        <v>46196.72965276291</v>
+        <v>46196.7296527662</v>
       </c>
     </row>
     <row r="17">
@@ -971,7 +971,7 @@
         </is>
       </c>
       <c r="H17" s="1" t="n">
-        <v>46196.72965276291</v>
+        <v>46196.7296527662</v>
       </c>
     </row>
     <row r="18">
@@ -999,7 +999,7 @@
         </is>
       </c>
       <c r="H18" s="1" t="n">
-        <v>46196.72965276291</v>
+        <v>46196.7296527662</v>
       </c>
     </row>
     <row r="19">
@@ -1031,7 +1031,579 @@
         </is>
       </c>
       <c r="H19" s="1" t="n">
-        <v>46196.72965276291</v>
+        <v>46196.7296527662</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>KSE100</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>179919.27</v>
+      </c>
+      <c r="C20" t="n">
+        <v>177931.32</v>
+      </c>
+      <c r="D20" t="n">
+        <v>179571.26</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1878.34</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>1.06%</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H20" s="1" t="n">
+        <v>46197.71990558558</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>KSE100PR</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>54864.73</v>
+      </c>
+      <c r="C21" t="n">
+        <v>54258.53</v>
+      </c>
+      <c r="D21" t="n">
+        <v>54758.61</v>
+      </c>
+      <c r="E21" t="n">
+        <v>572.78</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>1.06%</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H21" s="1" t="n">
+        <v>46197.71990558558</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>ALLSHR</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>108789.81</v>
+      </c>
+      <c r="C22" t="n">
+        <v>107660.45</v>
+      </c>
+      <c r="D22" t="n">
+        <v>108600.93</v>
+      </c>
+      <c r="E22" t="n">
+        <v>1073.54</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>1.00%</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H22" s="1" t="n">
+        <v>46197.71990558558</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>KSE30</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>53631.69</v>
+      </c>
+      <c r="C23" t="n">
+        <v>53056.2</v>
+      </c>
+      <c r="D23" t="n">
+        <v>53548.41</v>
+      </c>
+      <c r="E23" t="n">
+        <v>525.53</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>0.99%</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H23" s="1" t="n">
+        <v>46197.71990558558</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>KMI30</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>257179.58</v>
+      </c>
+      <c r="C24" t="n">
+        <v>254968.93</v>
+      </c>
+      <c r="D24" t="n">
+        <v>256725.69</v>
+      </c>
+      <c r="E24" t="n">
+        <v>1936.42</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>0.76%</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H24" s="1" t="n">
+        <v>46197.71990558558</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>BKTI</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>48822.72</v>
+      </c>
+      <c r="C25" t="n">
+        <v>47989.24</v>
+      </c>
+      <c r="D25" t="n">
+        <v>48625.03</v>
+      </c>
+      <c r="E25" t="n">
+        <v>658.39</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>1.37%</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H25" s="1" t="n">
+        <v>46197.71990558558</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>OGTI</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>37256.17</v>
+      </c>
+      <c r="C26" t="n">
+        <v>36819.41</v>
+      </c>
+      <c r="D26" t="n">
+        <v>37179.52</v>
+      </c>
+      <c r="E26" t="n">
+        <v>345.86</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>0.94%</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H26" s="1" t="n">
+        <v>46197.71990558558</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>KMIALLSHR</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>70743.5</v>
+      </c>
+      <c r="C27" t="n">
+        <v>70070.62</v>
+      </c>
+      <c r="D27" t="n">
+        <v>70620.69</v>
+      </c>
+      <c r="E27" t="n">
+        <v>683.55</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>0.98%</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H27" s="1" t="n">
+        <v>46197.71990558558</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>PSXDIV20</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>83080.73</v>
+      </c>
+      <c r="C28" t="n">
+        <v>82317.61</v>
+      </c>
+      <c r="D28" t="n">
+        <v>82793.49000000001</v>
+      </c>
+      <c r="E28" t="n">
+        <v>545.74</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>0.66%</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H28" s="1" t="n">
+        <v>46197.71990558558</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>UPP9</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>63136.26</v>
+      </c>
+      <c r="C29" t="n">
+        <v>62378.69</v>
+      </c>
+      <c r="D29" t="n">
+        <v>62995.45</v>
+      </c>
+      <c r="E29" t="n">
+        <v>666.12</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>1.07%</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H29" s="1" t="n">
+        <v>46197.71990558558</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>NITPGI</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>47434.28</v>
+      </c>
+      <c r="C30" t="n">
+        <v>46888.28</v>
+      </c>
+      <c r="D30" t="n">
+        <v>47359.99</v>
+      </c>
+      <c r="E30" t="n">
+        <v>505.54</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>1.08%</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H30" s="1" t="n">
+        <v>46197.71990558558</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>NBPPGI</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>51612.52</v>
+      </c>
+      <c r="C31" t="n">
+        <v>51069.45</v>
+      </c>
+      <c r="D31" t="n">
+        <v>51541.72</v>
+      </c>
+      <c r="E31" t="n">
+        <v>497.97</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>0.98%</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H31" s="1" t="n">
+        <v>46197.71990558558</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>MZNPI</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>31684.08</v>
+      </c>
+      <c r="C32" t="n">
+        <v>31377.86</v>
+      </c>
+      <c r="D32" t="n">
+        <v>31613.22</v>
+      </c>
+      <c r="E32" t="n">
+        <v>252.84</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>0.81%</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H32" s="1" t="n">
+        <v>46197.71990558558</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>JSMFI</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>43348.35</v>
+      </c>
+      <c r="C33" t="n">
+        <v>42738.98</v>
+      </c>
+      <c r="D33" t="n">
+        <v>43264.52</v>
+      </c>
+      <c r="E33" t="n">
+        <v>571.99</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>1.34%</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H33" s="1" t="n">
+        <v>46197.71990558558</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>ACI</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>24494.56</v>
+      </c>
+      <c r="C34" t="n">
+        <v>24171.51</v>
+      </c>
+      <c r="D34" t="n">
+        <v>24458.68</v>
+      </c>
+      <c r="E34" t="n">
+        <v>412.45</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>1.72%</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H34" s="1" t="n">
+        <v>46197.71990558558</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>JSGBKTI</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>74063.5</v>
+      </c>
+      <c r="C35" t="n">
+        <v>73006.11</v>
+      </c>
+      <c r="D35" t="n">
+        <v>73681.62</v>
+      </c>
+      <c r="E35" t="n">
+        <v>664.26</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>0.91%</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H35" s="1" t="n">
+        <v>46197.71990558558</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>HBLTTI</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="n">
+        <v>18601.61</v>
+      </c>
+      <c r="E36" t="n">
+        <v>5.65</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>0.03%</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H36" s="1" t="n">
+        <v>46197.71990558558</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>MII30</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>23511.75</v>
+      </c>
+      <c r="C37" t="n">
+        <v>23261.84</v>
+      </c>
+      <c r="D37" t="n">
+        <v>23461.72</v>
+      </c>
+      <c r="E37" t="n">
+        <v>225.93</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>0.97%</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H37" s="1" t="n">
+        <v>46197.71990558558</v>
       </c>
     </row>
   </sheetData>

</xml_diff>